<commit_message>
[Templates] Add 1 more Representative in Template
</commit_message>
<xml_diff>
--- a/backend/data_wizard/tests/templates/third_parties_ecosystem_template.xlsx
+++ b/backend/data_wizard/tests/templates/third_parties_ecosystem_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\backend\data_wizard\tests\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\product-docs\.gitbook\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4594D145-2EA5-4136-8421-0A8AC7FB8944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34F05CB7-C0F3-4439-B3AC-E28A7E3FBBFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4536" yWindow="2028" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Entities" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="84">
   <si>
     <t>ref_id</t>
   </si>
@@ -257,6 +257,24 @@
   </si>
   <si>
     <t>Compliance Manager</t>
+  </si>
+  <si>
+    <t>alexandre.morel@acmecorp.com</t>
+  </si>
+  <si>
+    <t>Alexandre</t>
+  </si>
+  <si>
+    <t>Morel</t>
+  </si>
+  <si>
+    <t>Primary operational contact for ACME Corporation security coordination</t>
+  </si>
+  <si>
+    <t>+33 1 42 00 00 03</t>
+  </si>
+  <si>
+    <t>Security Coordinator</t>
   </si>
 </sst>
 </file>
@@ -314,12 +332,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -996,13 +1015,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C56EDC4-5FDC-4B05-889D-1A302F57D200}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.88671875" customWidth="1"/>
-    <col min="4" max="4" width="44.109375" customWidth="1"/>
+    <col min="1" max="1" width="30" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="63.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.6640625" customWidth="1"/>
-    <col min="6" max="6" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="21.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1033,22 +1052,22 @@
       <c r="A2" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="3" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1056,22 +1075,45 @@
       <c r="A3" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1079,8 +1121,9 @@
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{7EC3EECF-D9E2-4361-AFAC-CAD1CE346FB9}"/>
     <hyperlink ref="A3" r:id="rId2" xr:uid="{B5BC6947-747D-4BFB-8830-F6C14A7D7631}"/>
+    <hyperlink ref="A4" r:id="rId3" xr:uid="{E7632B3E-F078-475A-8F2A-9BF8F35D95C4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[Templates] Fix Template Representatives Page Name
Remove useless space in front of the sheet name
</commit_message>
<xml_diff>
--- a/backend/data_wizard/tests/templates/third_parties_ecosystem_template.xlsx
+++ b/backend/data_wizard/tests/templates/third_parties_ecosystem_template.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\product-docs\.gitbook\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34F05CB7-C0F3-4439-B3AC-E28A7E3FBBFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75431463-6B77-4A0D-BA36-D11CF9755F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4536" yWindow="2028" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2880" yWindow="-11160" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Entities" sheetId="1" r:id="rId1"/>
     <sheet name="Solutions" sheetId="2" r:id="rId2"/>
     <sheet name="Contracts" sheetId="3" r:id="rId3"/>
-    <sheet name=" Representatives" sheetId="4" r:id="rId4"/>
+    <sheet name="Representatives" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>

</xml_diff>